<commit_message>
feat: add evaluation rubric prompt module
</commit_message>
<xml_diff>
--- a/data/evaluation_rubric/test_rubric.xlsx
+++ b/data/evaluation_rubric/test_rubric.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wang ngai wong\Desktop\Document\Research\Confidence Modeling\Code\Evaluation Agent\data\Evaluation Rubric\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wang ngai wong\Desktop\Document\Research\Confidence Modeling\Code\Evaluation Agent\data\evaluation_rubric\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{653527D9-86EC-4639-BB01-160018337DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{088D832C-8504-4813-BD17-54E7CD194E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3915" yWindow="405" windowWidth="21600" windowHeight="12510" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rubric" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
   <si>
     <t>Type</t>
   </si>
@@ -170,13 +170,84 @@
   </si>
   <si>
     <t>a Likert-scale approach is preferred due to its simplicity and ease of interpretation.</t>
+  </si>
+  <si>
+    <t>The evaluator assigns a score from 1 to 5 based on the descriptions of each attribute and the rubric.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The scores for the two types, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Potential Impact</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fidelity</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, are calculated based on the scores of their respective attributes. The weight assigned to each attribute is determined by the evaluator based on their own </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>concerns and attention</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -186,6 +257,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -699,7 +778,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A9DB0AB-65EA-4649-BC73-036C9F116FDB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.140625" bestFit="1" customWidth="1"/>
@@ -710,6 +789,16 @@
         <v>47</v>
       </c>
     </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>